<commit_message>
Add newest reading (Sep 6 5:17 PM, 220 mg/dL)
</commit_message>
<xml_diff>
--- a/blood_sugar_log.xlsx
+++ b/blood_sugar_log.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t xml:space="preserve">Date/Time</t>
   </si>
@@ -43,6 +43,9 @@
   </si>
   <si>
     <t xml:space="preserve">Post-meal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-06 17:17</t>
   </si>
   <si>
     <t xml:space="preserve">2026-09-07 17:16</t>
@@ -642,7 +645,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="4" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>6</v>
@@ -658,7 +661,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="4" t="n">
-        <v>252</v>
+        <v>200</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>6</v>
@@ -670,12 +673,18 @@
       <c r="E4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5"/>
+      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>252</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>6</v>
+      </c>
       <c r="D5" s="6" t="str">
         <f aca="false">IF(OR($B5="",$C5=""),"",IF(AND($B5&gt;=VLOOKUP($C5,Targets!$A$2:$C$5,2,FALSE()),$B5&lt;=VLOOKUP($C5,Targets!$A$2:$C$5,3,FALSE())),"In range",IF($B5&lt;VLOOKUP($C5,Targets!$A$2:$C$5,2,FALSE()),"Low","High")))</f>
-        <v/>
+        <v>High</v>
       </c>
       <c r="E5" s="4"/>
     </row>
@@ -5641,25 +5650,25 @@
     </row>
     <row r="504" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A504" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="505" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A505" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B505" s="7" t="n">
         <v>96</v>
       </c>
       <c r="C505" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D505" s="7" t="str">
         <f aca="false">IF(OR($B505="",$C505=""),"",IF(AND($B505&gt;=VLOOKUP($C505,Targets!$A$2:$C$5,2,FALSE()),$B505&lt;=VLOOKUP($C505,Targets!$A$2:$C$5,3,FALSE())),"In range",IF($B505&lt;VLOOKUP($C505,Targets!$A$2:$C$5,2,FALSE()),"Low","High")))</f>
         <v>In range</v>
       </c>
       <c r="E505" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -5707,15 +5716,15 @@
         <v>2</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="6" t="n">
         <v>80</v>
@@ -5737,7 +5746,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>80</v>
@@ -5748,7 +5757,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>90</v>
@@ -5759,7 +5768,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -5787,49 +5796,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B1" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="11" t="n">
         <f aca="false">COUNTIF(Log!B2:B501,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">IFERROR(AVERAGE(Log!B2:B501),"")</f>
-        <v>200.666666666667</v>
+        <v>205.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">IFERROR((B4+46.7)/28.7,"")</f>
-        <v>8.61904761904762</v>
+        <v>8.78745644599303</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">IFERROR(COUNTIF(Log!D2:D501,"In range")/COUNTIF(Log!B2:B501,"&lt;&gt;"),"")</f>
-        <v>0.333333333333333</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">COUNTIF(Log!B2:B501,"&lt;70")</f>
@@ -5838,7 +5847,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>

</xml_diff>

<commit_message>
Auto-rebuild blood_sugar_log.xlsx from data/readings.json
</commit_message>
<xml_diff>
--- a/blood_sugar_log.xlsx
+++ b/blood_sugar_log.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Targets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>